<commit_message>
Split up large CAS + quality checked version
</commit_message>
<xml_diff>
--- a/TestCAS.xlsx
+++ b/TestCAS.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/arche/Documents/Python/ARCHEscreeningTool/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1334209-E710-4242-A626-05B9143B807C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{950B1B3F-827F-9341-9CB2-F86997FC7BE1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28580" yWindow="1060" windowWidth="27720" windowHeight="17440" xr2:uid="{AC7C4B23-1DA4-2B48-871A-9902A8034EEE}"/>
   </bookViews>
@@ -162,7 +162,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -174,9 +174,6 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -535,47 +532,47 @@
       <c r="C2" s="4"/>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
+      <c r="A3" s="1" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
+      <c r="A4" s="1" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A5" t="s">
+      <c r="A5" s="1" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A6" t="s">
+      <c r="A6" s="1" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A7" t="s">
+      <c r="A7" s="1" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A8" t="s">
+      <c r="A8" s="1" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A9" s="5" t="s">
+      <c r="A9" s="1" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A10" t="s">
+      <c r="A10" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A11" t="s">
+      <c r="A11" s="1" t="s">
         <v>12</v>
       </c>
     </row>

</xml_diff>